<commit_message>
enemyDataLabel 의 act1 보스 이름 수정
일본어, 중국어 수정
</commit_message>
<xml_diff>
--- a/Assets/Resources/DataFiles/EnemyData/1. ExcelFile/EnemyDataLabel.xlsx
+++ b/Assets/Resources/DataFiles/EnemyData/1. ExcelFile/EnemyDataLabel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m\Desktop\Project2\Assets\Resources\DataFiles\EnemyData\1. ExcelFile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93E19C9B-6AC4-4C2A-863C-9EA0BF3BAAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA6B4F5-71FD-4DE2-8919-29CDC4B2551B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-17340" yWindow="1845" windowWidth="14745" windowHeight="12330" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KOR" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="47">
   <si>
     <t>enemyId</t>
   </si>
@@ -295,13 +295,6 @@
     <t>双足行走型机械</t>
   </si>
   <si>
-    <t>SpiderX</t>
-  </si>
-  <si>
-    <t>SpiderX</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <r>
       <t>移</t>
     </r>
@@ -351,6 +344,40 @@
   </si>
   <si>
     <t>Moving_coffer</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SPIDER X</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>スパイダ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ー</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>蜘蛛X</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -895,7 +922,7 @@
         <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.4">
@@ -903,7 +930,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.4">
@@ -911,7 +938,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.4">
@@ -919,7 +946,7 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.4">
@@ -927,7 +954,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.4">
@@ -935,7 +962,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.4">
@@ -943,7 +970,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.4">
@@ -951,7 +978,7 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.4">
@@ -959,7 +986,7 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1041,12 +1068,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:2" ht="18" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.4">
@@ -1054,7 +1081,7 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1141,7 +1168,7 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.4">
@@ -1149,7 +1176,7 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>